<commit_message>
[Infra] - Added 'CXXFLAGS += -DDISABLE_MSHR' [perf. study] - Added MSHR related config.
</commit_message>
<xml_diff>
--- a/perf_study/plot/overall_perf_study.xlsx
+++ b/perf_study/plot/overall_perf_study.xlsx
@@ -40,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8D0D0"/>
+        <fgColor rgb="FFD4F5D4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD4F5D4"/>
+        <fgColor rgb="FFF8D0D0"/>
       </patternFill>
     </fill>
   </fills>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,16 @@
           <t>MSHR_MERGE_ENTRY_FAIL</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MSHR_ENTRY_FAIL</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>LINE_ALLOC_FAIL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,106 +489,136 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>60.960</t>
+          <t>29.871</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>15.843</t>
+          <t>5.756</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>14553.780</t>
+          <t>12066.066</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>3671.740</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>1476.818</t>
+          <t>13170.246</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>12.146</t>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>0.864</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>default-cfg-11-25-eve</t>
+          <t>regress_disable_mshr_l2_correlation</t>
         </is>
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>60.960 (+0.000%)</t>
+          <t>29.871 (+0.000%)</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>15.843 (+0.000%)</t>
+          <t>5.756 (+0.000%)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>14553.780 (+0.000%)</t>
+          <t>12066.066 (+0.000%)</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t>3671.740 (+0.000%)</t>
+          <t>0.000 (+0.000%)</t>
         </is>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
-          <t>1476.818 (+0.000%)</t>
+          <t>13170.246 (+0.000%)</t>
         </is>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t>12.146 (+0.000%)</t>
+          <t>0.000 (+0.000%)</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>0.000 (+0.000%)</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>0.864 (+0.000%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>l2_max_merge_zero</t>
+          <t>regress_enable_mshr_l2_correlation</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>60.342 (-1.013%)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>15.683 (-1.013%)</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>14553.780 (+0.000%)</t>
+          <t>34.293 (+14.801%)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>4.628 (-19.594%)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>8536.831 (-29.249%)</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>3671.740 (+0.000%)</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1810.607 (+22.602%)</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>13.647 (+12.356%)</t>
+          <t>3577.276 (-72.838%)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>146.261 (+inf%)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>7.180 (+inf%)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>1.647 (+90.605%)</t>
         </is>
       </c>
     </row>

</xml_diff>